<commit_message>
fix(v3): bump GNSS ECO board revision to V3.7
</commit_message>
<xml_diff>
--- a/hardware/expansion-board-v3/CHECKLIST.xlsx
+++ b/hardware/expansion-board-v3/CHECKLIST.xlsx
@@ -7,10 +7,10 @@
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet name="V3.4 核对清单" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet name="V3.7 核对清单" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm.Print_Titles" localSheetId="0">'V3.4 核对清单'!$1:$1</definedName>
+    <definedName name="_xlnm.Print_Titles" localSheetId="0">'V3.7 核对清单'!$1:$1</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -504,7 +504,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
-  <dimension ref="A1:G172"/>
+  <dimension ref="A1:G173"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="6" customWidth="1" min="1" max="1"/>
@@ -1814,7 +1814,7 @@
       </c>
       <c r="E44" s="2" t="inlineStr">
         <is>
-          <t>55.6, 79.9</t>
+          <t>55.6, 80.1</t>
         </is>
       </c>
       <c r="F44" s="4" t="inlineStr">
@@ -1843,7 +1843,7 @@
       </c>
       <c r="E45" s="2" t="inlineStr">
         <is>
-          <t>55.6, 84.5</t>
+          <t>55.6, 85.2</t>
         </is>
       </c>
       <c r="F45" s="4" t="inlineStr">
@@ -1901,7 +1901,7 @@
       </c>
       <c r="E47" s="2" t="inlineStr">
         <is>
-          <t>110.9, 62.1</t>
+          <t>110.2, 61.2</t>
         </is>
       </c>
       <c r="F47" s="4" t="inlineStr">
@@ -2017,7 +2017,7 @@
       </c>
       <c r="E51" s="2" t="inlineStr">
         <is>
-          <t>76.2, 55.1</t>
+          <t>63.4, 63.3</t>
         </is>
       </c>
       <c r="F51" s="4" t="inlineStr">
@@ -2046,7 +2046,7 @@
       </c>
       <c r="E52" s="2" t="inlineStr">
         <is>
-          <t>78.9, 55.1</t>
+          <t>56.5, 64.6</t>
         </is>
       </c>
       <c r="F52" s="4" t="inlineStr">
@@ -2075,7 +2075,7 @@
       </c>
       <c r="E53" s="2" t="inlineStr">
         <is>
-          <t>81.5, 55.1</t>
+          <t>56.3, 62.4</t>
         </is>
       </c>
       <c r="F53" s="4" t="inlineStr">
@@ -2946,7 +2946,7 @@
       </c>
       <c r="E84" s="2" t="inlineStr">
         <is>
-          <t>95.4, 66.6</t>
+          <t>58.8, 76.4</t>
         </is>
       </c>
       <c r="F84" s="4" t="inlineStr">
@@ -2975,7 +2975,7 @@
       </c>
       <c r="E85" s="2" t="inlineStr">
         <is>
-          <t>83.6, 71.2</t>
+          <t>61.8, 73.3</t>
         </is>
       </c>
       <c r="F85" s="4" t="inlineStr">
@@ -3153,7 +3153,7 @@
       </c>
       <c r="E91" s="2" t="inlineStr">
         <is>
-          <t>55.6, 82.3</t>
+          <t>55.6, 82.6</t>
         </is>
       </c>
       <c r="F91" s="4" t="inlineStr">
@@ -3212,7 +3212,7 @@
       </c>
       <c r="E94" s="2" t="inlineStr">
         <is>
-          <t>92.1, 62.1</t>
+          <t>61.8, 64.8</t>
         </is>
       </c>
       <c r="F94" s="4" t="inlineStr">
@@ -3477,7 +3477,7 @@
       </c>
       <c r="E103" s="2" t="inlineStr">
         <is>
-          <t>92.1, 66.6</t>
+          <t>58.0, 67.6</t>
         </is>
       </c>
       <c r="F103" s="4" t="inlineStr">
@@ -3665,7 +3665,7 @@
       </c>
       <c r="E111" s="2" t="inlineStr">
         <is>
-          <t>88.5, 62.1</t>
+          <t>61.8, 67.4</t>
         </is>
       </c>
       <c r="F111" s="4" t="inlineStr">
@@ -3694,7 +3694,7 @@
       </c>
       <c r="E112" s="2" t="inlineStr">
         <is>
-          <t>88.6, 66.6</t>
+          <t>56.4, 69.7</t>
         </is>
       </c>
       <c r="F112" s="4" t="inlineStr">
@@ -3782,7 +3782,7 @@
       </c>
       <c r="E116" s="2" t="inlineStr">
         <is>
-          <t>84.0, 62.1</t>
+          <t>61.8, 70.2</t>
         </is>
       </c>
       <c r="F116" s="4" t="inlineStr">
@@ -3811,7 +3811,7 @@
       </c>
       <c r="E117" s="2" t="inlineStr">
         <is>
-          <t>84.0, 66.6</t>
+          <t>57.8, 72.6</t>
         </is>
       </c>
       <c r="F117" s="4" t="inlineStr">
@@ -4365,7 +4365,7 @@
       </c>
       <c r="E135" s="14" t="inlineStr">
         <is>
-          <t>73.0, 55.1</t>
+          <t>58.8, 63.3</t>
         </is>
       </c>
       <c r="F135" s="16" t="inlineStr">
@@ -4591,7 +4591,7 @@
       </c>
       <c r="E145" s="2" t="inlineStr">
         <is>
-          <t>68.0, 54.5</t>
+          <t>52.9, 74.1</t>
         </is>
       </c>
       <c r="F145" s="4" t="inlineStr">
@@ -4692,244 +4692,244 @@
       <c r="A149" s="2" t="inlineStr"/>
       <c r="B149" s="3" t="inlineStr">
         <is>
+          <t>J7</t>
+        </is>
+      </c>
+      <c r="C149" s="4" t="inlineStr">
+        <is>
+          <t>U.FL_IFA_TEST(π后调试口)</t>
+        </is>
+      </c>
+      <c r="D149" s="4" t="inlineStr">
+        <is>
+          <t>U.FL_Hirose_U.FL-R-SMT-1_Vertical</t>
+        </is>
+      </c>
+      <c r="E149" s="2" t="inlineStr">
+        <is>
+          <t>103.1, 61.3</t>
+        </is>
+      </c>
+      <c r="F149" s="4" t="inlineStr">
+        <is>
+          <t>E 1090 接收链</t>
+        </is>
+      </c>
+      <c r="G149" s="5" t="inlineStr"/>
+    </row>
+    <row r="150" ht="19" customHeight="1">
+      <c r="A150" s="2" t="inlineStr"/>
+      <c r="B150" s="3" t="inlineStr">
+        <is>
           <t>J8</t>
         </is>
       </c>
-      <c r="C149" s="4" t="inlineStr">
+      <c r="C150" s="4" t="inlineStr">
         <is>
           <t>U.FL→内置patch</t>
         </is>
       </c>
-      <c r="D149" s="4" t="inlineStr">
+      <c r="D150" s="4" t="inlineStr">
         <is>
           <t>U.FL_Hirose_U.FL-R-SMT-1_Vertical</t>
         </is>
       </c>
-      <c r="E149" s="2" t="inlineStr">
-        <is>
-          <t>60.0, 54.5</t>
-        </is>
-      </c>
-      <c r="F149" s="4" t="inlineStr">
+      <c r="E150" s="2" t="inlineStr">
+        <is>
+          <t>52.9, 64.4</t>
+        </is>
+      </c>
+      <c r="F150" s="4" t="inlineStr">
         <is>
           <t>C 传感器 + GNSS</t>
         </is>
       </c>
-      <c r="G149" s="5" t="inlineStr"/>
-    </row>
-    <row r="150" ht="19" customHeight="1"/>
-    <row r="151" ht="19" customHeight="1">
-      <c r="A151" s="10" t="inlineStr"/>
-      <c r="B151" s="11" t="inlineStr">
+      <c r="G150" s="5" t="inlineStr"/>
+    </row>
+    <row r="151" ht="19" customHeight="1"/>
+    <row r="152" ht="19" customHeight="1">
+      <c r="A152" s="10" t="inlineStr"/>
+      <c r="B152" s="11" t="inlineStr">
         <is>
           <t>ANT1</t>
         </is>
       </c>
-      <c r="C151" s="12" t="inlineStr">
+      <c r="C152" s="12" t="inlineStr">
         <is>
           <t>IFA_1090</t>
         </is>
       </c>
-      <c r="D151" s="12" t="inlineStr">
+      <c r="D152" s="12" t="inlineStr">
         <is>
           <t>ANT_IFA_1090MHz</t>
         </is>
       </c>
-      <c r="E151" s="10" t="inlineStr">
-        <is>
-          <t>102.0, 57.8</t>
-        </is>
-      </c>
-      <c r="F151" s="12" t="inlineStr">
+      <c r="E152" s="10" t="inlineStr">
+        <is>
+          <t>85.5, 57.8</t>
+        </is>
+      </c>
+      <c r="F152" s="12" t="inlineStr">
         <is>
           <t>不贴（板载天线）</t>
         </is>
       </c>
-      <c r="G151" s="13" t="inlineStr"/>
-    </row>
-    <row r="152" ht="19" customHeight="1"/>
-    <row r="153" ht="19" customHeight="1">
-      <c r="A153" s="10" t="inlineStr"/>
-      <c r="B153" s="11" t="inlineStr">
-        <is>
-          <t>ZP1</t>
-        </is>
-      </c>
-      <c r="C153" s="12" t="inlineStr">
-        <is>
-          <t>DNP 并-天线侧</t>
-        </is>
-      </c>
-      <c r="D153" s="12" t="inlineStr">
-        <is>
-          <t>C_0603_1608Metric</t>
-        </is>
-      </c>
-      <c r="E153" s="10" t="inlineStr">
-        <is>
-          <t>105.3, 58.2</t>
-        </is>
-      </c>
-      <c r="F153" s="12" t="inlineStr">
-        <is>
-          <t>不贴（DNP）</t>
-        </is>
-      </c>
-      <c r="G153" s="13" t="inlineStr"/>
-    </row>
+      <c r="G152" s="13" t="inlineStr"/>
+    </row>
+    <row r="153" ht="19" customHeight="1"/>
     <row r="154" ht="19" customHeight="1">
       <c r="A154" s="10" t="inlineStr"/>
       <c r="B154" s="11" t="inlineStr">
         <is>
+          <t>ZP1</t>
+        </is>
+      </c>
+      <c r="C154" s="12" t="inlineStr">
+        <is>
+          <t>DNP 并-天线侧</t>
+        </is>
+      </c>
+      <c r="D154" s="12" t="inlineStr">
+        <is>
+          <t>C_0603_1608Metric</t>
+        </is>
+      </c>
+      <c r="E154" s="10" t="inlineStr">
+        <is>
+          <t>85.5, 63.6</t>
+        </is>
+      </c>
+      <c r="F154" s="12" t="inlineStr">
+        <is>
+          <t>不贴（DNP）</t>
+        </is>
+      </c>
+      <c r="G154" s="13" t="inlineStr"/>
+    </row>
+    <row r="155" ht="19" customHeight="1">
+      <c r="A155" s="10" t="inlineStr"/>
+      <c r="B155" s="11" t="inlineStr">
+        <is>
           <t>ZP2</t>
         </is>
       </c>
-      <c r="C154" s="12" t="inlineStr">
+      <c r="C155" s="12" t="inlineStr">
         <is>
           <t>DNP 并-电台侧</t>
         </is>
       </c>
-      <c r="D154" s="12" t="inlineStr">
+      <c r="D155" s="12" t="inlineStr">
         <is>
           <t>C_0603_1608Metric</t>
         </is>
       </c>
-      <c r="E154" s="10" t="inlineStr">
-        <is>
-          <t>108.1, 62.1</t>
-        </is>
-      </c>
-      <c r="F154" s="12" t="inlineStr">
+      <c r="E155" s="10" t="inlineStr">
+        <is>
+          <t>90.5, 63.6</t>
+        </is>
+      </c>
+      <c r="F155" s="12" t="inlineStr">
         <is>
           <t>不贴（DNP）</t>
         </is>
       </c>
-      <c r="G154" s="13" t="inlineStr"/>
-    </row>
-    <row r="155" ht="19" customHeight="1"/>
-    <row r="156" ht="19" customHeight="1">
-      <c r="A156" s="2" t="inlineStr"/>
-      <c r="B156" s="3" t="inlineStr">
+      <c r="G155" s="13" t="inlineStr"/>
+    </row>
+    <row r="156" ht="19" customHeight="1"/>
+    <row r="157" ht="19" customHeight="1">
+      <c r="A157" s="2" t="inlineStr"/>
+      <c r="B157" s="3" t="inlineStr">
         <is>
           <t>ZS1</t>
         </is>
       </c>
-      <c r="C156" s="4" t="inlineStr">
+      <c r="C157" s="4" t="inlineStr">
         <is>
           <t>0R 串</t>
         </is>
       </c>
-      <c r="D156" s="4" t="inlineStr">
+      <c r="D157" s="4" t="inlineStr">
         <is>
           <t>L_0603_1608Metric</t>
         </is>
       </c>
-      <c r="E156" s="2" t="inlineStr">
-        <is>
-          <t>104.3, 62.1</t>
-        </is>
-      </c>
-      <c r="F156" s="4" t="inlineStr">
+      <c r="E157" s="2" t="inlineStr">
+        <is>
+          <t>88.0, 62.9</t>
+        </is>
+      </c>
+      <c r="F157" s="4" t="inlineStr">
         <is>
           <t>E 1090 接收链</t>
         </is>
       </c>
-      <c r="G156" s="5" t="inlineStr"/>
-    </row>
-    <row r="157" ht="19" customHeight="1"/>
-    <row r="158" ht="19" customHeight="1">
-      <c r="A158" s="10" t="inlineStr"/>
-      <c r="B158" s="11" t="inlineStr">
-        <is>
-          <t>SW1</t>
-        </is>
-      </c>
-      <c r="C158" s="12" t="inlineStr">
-        <is>
-          <t>RESET短接焊盘</t>
-        </is>
-      </c>
-      <c r="D158" s="12" t="inlineStr">
-        <is>
-          <t>SolderJumper-2_P1.3mm_Open_Pad1.0x1.5mm</t>
-        </is>
-      </c>
-      <c r="E158" s="10" t="inlineStr">
-        <is>
-          <t>88.7, 91.3</t>
-        </is>
-      </c>
-      <c r="F158" s="12" t="inlineStr">
-        <is>
-          <t>不贴（短接焊盘）</t>
-        </is>
-      </c>
-      <c r="G158" s="13" t="inlineStr"/>
-    </row>
+      <c r="G157" s="5" t="inlineStr"/>
+    </row>
+    <row r="158" ht="19" customHeight="1"/>
     <row r="159" ht="19" customHeight="1">
       <c r="A159" s="10" t="inlineStr"/>
       <c r="B159" s="11" t="inlineStr">
         <is>
+          <t>SW1</t>
+        </is>
+      </c>
+      <c r="C159" s="12" t="inlineStr">
+        <is>
+          <t>RESET短接焊盘</t>
+        </is>
+      </c>
+      <c r="D159" s="12" t="inlineStr">
+        <is>
+          <t>SolderJumper-2_P1.3mm_Open_Pad1.0x1.5mm</t>
+        </is>
+      </c>
+      <c r="E159" s="10" t="inlineStr">
+        <is>
+          <t>88.7, 91.3</t>
+        </is>
+      </c>
+      <c r="F159" s="12" t="inlineStr">
+        <is>
+          <t>不贴（短接焊盘）</t>
+        </is>
+      </c>
+      <c r="G159" s="13" t="inlineStr"/>
+    </row>
+    <row r="160" ht="19" customHeight="1">
+      <c r="A160" s="10" t="inlineStr"/>
+      <c r="B160" s="11" t="inlineStr">
+        <is>
           <t>SW2</t>
         </is>
       </c>
-      <c r="C159" s="12" t="inlineStr">
+      <c r="C160" s="12" t="inlineStr">
         <is>
           <t>BOOTSEL短接焊盘</t>
         </is>
       </c>
-      <c r="D159" s="12" t="inlineStr">
+      <c r="D160" s="12" t="inlineStr">
         <is>
           <t>SolderJumper-2_P1.3mm_Open_Pad1.0x1.5mm</t>
         </is>
       </c>
-      <c r="E159" s="10" t="inlineStr">
+      <c r="E160" s="10" t="inlineStr">
         <is>
           <t>92.9, 91.3</t>
         </is>
       </c>
-      <c r="F159" s="12" t="inlineStr">
+      <c r="F160" s="12" t="inlineStr">
         <is>
           <t>不贴（短接焊盘）</t>
         </is>
       </c>
-      <c r="G159" s="13" t="inlineStr"/>
-    </row>
-    <row r="160" ht="19" customHeight="1"/>
-    <row r="161" ht="19" customHeight="1">
-      <c r="A161" s="10" t="inlineStr"/>
-      <c r="B161" s="11" t="inlineStr">
-        <is>
-          <t>TP1</t>
-        </is>
-      </c>
-      <c r="C161" s="12" t="inlineStr">
-        <is>
-          <t>TestPoint</t>
-        </is>
-      </c>
-      <c r="D161" s="12" t="inlineStr">
-        <is>
-          <t>TestPoint_Pad_1.0x1.0mm</t>
-        </is>
-      </c>
-      <c r="E161" s="10" t="inlineStr">
-        <is>
-          <t>102.0, 91.3</t>
-        </is>
-      </c>
-      <c r="F161" s="12" t="inlineStr">
-        <is>
-          <t>不贴（测试点焊盘）</t>
-        </is>
-      </c>
-      <c r="G161" s="13" t="inlineStr"/>
-    </row>
+      <c r="G160" s="13" t="inlineStr"/>
+    </row>
+    <row r="161" ht="19" customHeight="1"/>
     <row r="162" ht="19" customHeight="1">
       <c r="A162" s="10" t="inlineStr"/>
       <c r="B162" s="11" t="inlineStr">
         <is>
-          <t>TP2</t>
+          <t>TP1</t>
         </is>
       </c>
       <c r="C162" s="12" t="inlineStr">
@@ -4944,7 +4944,7 @@
       </c>
       <c r="E162" s="10" t="inlineStr">
         <is>
-          <t>104.9, 91.3</t>
+          <t>102.0, 91.3</t>
         </is>
       </c>
       <c r="F162" s="12" t="inlineStr">
@@ -4958,7 +4958,7 @@
       <c r="A163" s="10" t="inlineStr"/>
       <c r="B163" s="11" t="inlineStr">
         <is>
-          <t>TP3</t>
+          <t>TP2</t>
         </is>
       </c>
       <c r="C163" s="12" t="inlineStr">
@@ -4973,7 +4973,7 @@
       </c>
       <c r="E163" s="10" t="inlineStr">
         <is>
-          <t>107.8, 91.3</t>
+          <t>104.9, 91.3</t>
         </is>
       </c>
       <c r="F163" s="12" t="inlineStr">
@@ -4987,7 +4987,7 @@
       <c r="A164" s="10" t="inlineStr"/>
       <c r="B164" s="11" t="inlineStr">
         <is>
-          <t>TP4</t>
+          <t>TP3</t>
         </is>
       </c>
       <c r="C164" s="12" t="inlineStr">
@@ -5002,7 +5002,7 @@
       </c>
       <c r="E164" s="10" t="inlineStr">
         <is>
-          <t>110.7, 91.3</t>
+          <t>107.8, 91.3</t>
         </is>
       </c>
       <c r="F164" s="12" t="inlineStr">
@@ -5016,7 +5016,7 @@
       <c r="A165" s="10" t="inlineStr"/>
       <c r="B165" s="11" t="inlineStr">
         <is>
-          <t>TP5</t>
+          <t>TP4</t>
         </is>
       </c>
       <c r="C165" s="12" t="inlineStr">
@@ -5031,7 +5031,7 @@
       </c>
       <c r="E165" s="10" t="inlineStr">
         <is>
-          <t>113.5, 91.3</t>
+          <t>110.7, 91.3</t>
         </is>
       </c>
       <c r="F165" s="12" t="inlineStr">
@@ -5045,7 +5045,7 @@
       <c r="A166" s="10" t="inlineStr"/>
       <c r="B166" s="11" t="inlineStr">
         <is>
-          <t>TP6</t>
+          <t>TP5</t>
         </is>
       </c>
       <c r="C166" s="12" t="inlineStr">
@@ -5060,7 +5060,7 @@
       </c>
       <c r="E166" s="10" t="inlineStr">
         <is>
-          <t>116.4, 91.3</t>
+          <t>113.5, 91.3</t>
         </is>
       </c>
       <c r="F166" s="12" t="inlineStr">
@@ -5074,66 +5074,66 @@
       <c r="A167" s="10" t="inlineStr"/>
       <c r="B167" s="11" t="inlineStr">
         <is>
+          <t>TP6</t>
+        </is>
+      </c>
+      <c r="C167" s="12" t="inlineStr">
+        <is>
+          <t>TestPoint</t>
+        </is>
+      </c>
+      <c r="D167" s="12" t="inlineStr">
+        <is>
+          <t>TestPoint_Pad_1.0x1.0mm</t>
+        </is>
+      </c>
+      <c r="E167" s="10" t="inlineStr">
+        <is>
+          <t>116.4, 91.3</t>
+        </is>
+      </c>
+      <c r="F167" s="12" t="inlineStr">
+        <is>
+          <t>不贴（测试点焊盘）</t>
+        </is>
+      </c>
+      <c r="G167" s="13" t="inlineStr"/>
+    </row>
+    <row r="168" ht="19" customHeight="1">
+      <c r="A168" s="10" t="inlineStr"/>
+      <c r="B168" s="11" t="inlineStr">
+        <is>
           <t>TP7</t>
         </is>
       </c>
-      <c r="C167" s="12" t="inlineStr">
+      <c r="C168" s="12" t="inlineStr">
         <is>
           <t>TestPoint</t>
         </is>
       </c>
-      <c r="D167" s="12" t="inlineStr">
+      <c r="D168" s="12" t="inlineStr">
         <is>
           <t>TestPoint_Pad_1.0x1.0mm</t>
         </is>
       </c>
-      <c r="E167" s="10" t="inlineStr">
+      <c r="E168" s="10" t="inlineStr">
         <is>
           <t>83.3, 95.2</t>
         </is>
       </c>
-      <c r="F167" s="12" t="inlineStr">
+      <c r="F168" s="12" t="inlineStr">
         <is>
           <t>不贴（测试点焊盘）</t>
         </is>
       </c>
-      <c r="G167" s="13" t="inlineStr"/>
-    </row>
-    <row r="168" ht="19" customHeight="1"/>
-    <row r="169" ht="19" customHeight="1">
-      <c r="A169" s="10" t="inlineStr"/>
-      <c r="B169" s="11" t="inlineStr">
-        <is>
-          <t>H1</t>
-        </is>
-      </c>
-      <c r="C169" s="12" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="D169" s="12" t="inlineStr">
-        <is>
-          <t>MountingHole_2.7mm_M2.5</t>
-        </is>
-      </c>
-      <c r="E169" s="10" t="inlineStr">
-        <is>
-          <t>54.0, 56.0</t>
-        </is>
-      </c>
-      <c r="F169" s="12" t="inlineStr">
-        <is>
-          <t>不贴（安装孔）</t>
-        </is>
-      </c>
-      <c r="G169" s="13" t="inlineStr"/>
-    </row>
+      <c r="G168" s="13" t="inlineStr"/>
+    </row>
+    <row r="169" ht="19" customHeight="1"/>
     <row r="170" ht="19" customHeight="1">
       <c r="A170" s="10" t="inlineStr"/>
       <c r="B170" s="11" t="inlineStr">
         <is>
-          <t>H2</t>
+          <t>H1</t>
         </is>
       </c>
       <c r="C170" s="12" t="inlineStr">
@@ -5148,7 +5148,7 @@
       </c>
       <c r="E170" s="10" t="inlineStr">
         <is>
-          <t>146.0, 56.0</t>
+          <t>54.0, 56.0</t>
         </is>
       </c>
       <c r="F170" s="12" t="inlineStr">
@@ -5162,7 +5162,7 @@
       <c r="A171" s="10" t="inlineStr"/>
       <c r="B171" s="11" t="inlineStr">
         <is>
-          <t>H3</t>
+          <t>H2</t>
         </is>
       </c>
       <c r="C171" s="12" t="inlineStr">
@@ -5177,7 +5177,7 @@
       </c>
       <c r="E171" s="10" t="inlineStr">
         <is>
-          <t>54.0, 106.0</t>
+          <t>146.0, 56.0</t>
         </is>
       </c>
       <c r="F171" s="12" t="inlineStr">
@@ -5191,30 +5191,59 @@
       <c r="A172" s="10" t="inlineStr"/>
       <c r="B172" s="11" t="inlineStr">
         <is>
+          <t>H3</t>
+        </is>
+      </c>
+      <c r="C172" s="12" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="D172" s="12" t="inlineStr">
+        <is>
+          <t>MountingHole_2.7mm_M2.5</t>
+        </is>
+      </c>
+      <c r="E172" s="10" t="inlineStr">
+        <is>
+          <t>54.0, 106.0</t>
+        </is>
+      </c>
+      <c r="F172" s="12" t="inlineStr">
+        <is>
+          <t>不贴（安装孔）</t>
+        </is>
+      </c>
+      <c r="G172" s="13" t="inlineStr"/>
+    </row>
+    <row r="173" ht="19" customHeight="1">
+      <c r="A173" s="10" t="inlineStr"/>
+      <c r="B173" s="11" t="inlineStr">
+        <is>
           <t>H4</t>
         </is>
       </c>
-      <c r="C172" s="12" t="inlineStr">
+      <c r="C173" s="12" t="inlineStr">
         <is>
           <t>—</t>
         </is>
       </c>
-      <c r="D172" s="12" t="inlineStr">
+      <c r="D173" s="12" t="inlineStr">
         <is>
           <t>MountingHole_2.7mm_M2.5</t>
         </is>
       </c>
-      <c r="E172" s="10" t="inlineStr">
+      <c r="E173" s="10" t="inlineStr">
         <is>
           <t>146.0, 106.0</t>
         </is>
       </c>
-      <c r="F172" s="12" t="inlineStr">
+      <c r="F173" s="12" t="inlineStr">
         <is>
           <t>不贴（安装孔）</t>
         </is>
       </c>
-      <c r="G172" s="13" t="inlineStr"/>
+      <c r="G173" s="13" t="inlineStr"/>
     </row>
   </sheetData>
   <printOptions gridLines="0"/>

</xml_diff>